<commit_message>
Complete problem 1 modeling pipeline and outputs
</commit_message>
<xml_diff>
--- a/A_MAGE_R3/output/tables/appendix1_features_normalized.xlsx
+++ b/A_MAGE_R3/output/tables/appendix1_features_normalized.xlsx
@@ -272,16 +272,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -297,7 +289,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -305,30 +297,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -627,76 +601,76 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:24">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -726,13 +700,13 @@
         <v>1</v>
       </c>
       <c r="I2">
-        <v>0.08578570437666902</v>
+        <v>0.02411167512690355</v>
       </c>
       <c r="J2">
         <v>0.5253611333291848</v>
       </c>
       <c r="K2">
-        <v>0.03817042329266983</v>
+        <v>0.06702573309395571</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -800,13 +774,13 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0.1139760287716643</v>
+        <v>0.0759493670886076</v>
       </c>
       <c r="J3">
         <v>0.3155362202257168</v>
       </c>
       <c r="K3">
-        <v>0.289571510474108</v>
+        <v>0.1587967820916404</v>
       </c>
       <c r="L3">
         <v>1</v>
@@ -874,7 +848,7 @@
         <v>0.4</v>
       </c>
       <c r="I4">
-        <v>0.1175779437675482</v>
+        <v>0.07716049382716049</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -945,7 +919,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.116003797433032</v>
+        <v>0.02137546468401487</v>
       </c>
       <c r="J5">
         <v>0.5748134894000466</v>
@@ -1016,7 +990,7 @@
         <v>1</v>
       </c>
       <c r="I6">
-        <v>0.5041997861457171</v>
+        <v>0.07815442561205273</v>
       </c>
       <c r="J6">
         <v>0.04613019951628614</v>
@@ -1090,7 +1064,7 @@
         <v>0.3271607529530718</v>
       </c>
       <c r="K7">
-        <v>0.06407886870780183</v>
+        <v>0.009909909909909909</v>
       </c>
       <c r="L7">
         <v>1</v>
@@ -1158,7 +1132,7 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.03532952907749563</v>
+        <v>0.03778558875219683</v>
       </c>
       <c r="J8">
         <v>0.1184414197886142</v>
@@ -1229,7 +1203,7 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>0.03420382186377766</v>
+        <v>0.01658374792703151</v>
       </c>
       <c r="J9">
         <v>0.06756725639203094</v>
@@ -1300,13 +1274,13 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="I10">
-        <v>0.05209803732565371</v>
+        <v>0.03761755485893417</v>
       </c>
       <c r="J10">
         <v>0.4353614449441348</v>
       </c>
       <c r="K10">
-        <v>0.08612887409003074</v>
+        <v>0.06457367106671423</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -1374,7 +1348,7 @@
         <v>1</v>
       </c>
       <c r="I11">
-        <v>0.1881086269824473</v>
+        <v>0.1028128031037827</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -1448,7 +1422,7 @@
         <v>0.2314430679987416</v>
       </c>
       <c r="K12">
-        <v>0.06318334564736415</v>
+        <v>0.08065595716198126</v>
       </c>
       <c r="L12">
         <v>0.5</v>
@@ -1519,7 +1493,7 @@
         <v>0.1211018776803749</v>
       </c>
       <c r="K13">
-        <v>0.1661138354812506</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="L13">
         <v>0.25</v>
@@ -1655,7 +1629,7 @@
         <v>1</v>
       </c>
       <c r="I15">
-        <v>0.3569509876362737</v>
+        <v>0.08413055711873944</v>
       </c>
       <c r="J15">
         <v>0.3452132711399759</v>
@@ -1726,13 +1700,13 @@
         <v>1</v>
       </c>
       <c r="I16">
-        <v>0.2616678217159539</v>
+        <v>0.03080939947780679</v>
       </c>
       <c r="J16">
         <v>0.2519146597290652</v>
       </c>
       <c r="K16">
-        <v>0.08228842164171955</v>
+        <v>0.08543380206951447</v>
       </c>
       <c r="L16">
         <v>0.75</v>
@@ -1800,13 +1774,13 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>0.1377745717244618</v>
+        <v>0.02070484581497797</v>
       </c>
       <c r="J17">
         <v>0.7637734129146833</v>
       </c>
       <c r="K17">
-        <v>0.1422067857495224</v>
+        <v>0.08157894736842106</v>
       </c>
       <c r="L17">
         <v>0.5</v>
@@ -1874,7 +1848,7 @@
         <v>0.5</v>
       </c>
       <c r="I18">
-        <v>0.1412917366279049</v>
+        <v>0.04539877300613497</v>
       </c>
       <c r="J18">
         <v>0.2248070949474241</v>
@@ -2013,7 +1987,7 @@
         <v>1</v>
       </c>
       <c r="I20">
-        <v>0.009468284781685644</v>
+        <v>0.005591798695246971</v>
       </c>
       <c r="J20">
         <v>0.4285149821768447</v>
@@ -2084,7 +2058,7 @@
         <v>1</v>
       </c>
       <c r="I21">
-        <v>0.195715352509112</v>
+        <v>0.07626310772163966</v>
       </c>
       <c r="J21">
         <v>0.6804572290040132</v>
@@ -2158,7 +2132,7 @@
         <v>0.4625338761141594</v>
       </c>
       <c r="K22">
-        <v>0.03597946542226411</v>
+        <v>0.03433098591549296</v>
       </c>
       <c r="L22">
         <v>1</v>
@@ -2226,13 +2200,13 @@
         <v>1</v>
       </c>
       <c r="I23">
-        <v>0.1848573968269061</v>
+        <v>0.04118050789293068</v>
       </c>
       <c r="J23">
         <v>0.5666867955757565</v>
       </c>
       <c r="K23">
-        <v>0.004369916782783756</v>
+        <v>0.01071428571428571</v>
       </c>
       <c r="L23">
         <v>0.5</v>
@@ -2300,13 +2274,13 @@
         <v>0</v>
       </c>
       <c r="I24">
-        <v>0.1285869752960457</v>
+        <v>0.06751592356687898</v>
       </c>
       <c r="J24">
         <v>0.4954078772013043</v>
       </c>
       <c r="K24">
-        <v>0.09272482582954525</v>
+        <v>0.06038756196484903</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -2374,13 +2348,13 @@
         <v>0</v>
       </c>
       <c r="I25">
-        <v>0.05187871893800355</v>
+        <v>0.04013377926421405</v>
       </c>
       <c r="J25">
         <v>0.03397318374409214</v>
       </c>
       <c r="K25">
-        <v>0.2068692012809782</v>
+        <v>0.09637404580152671</v>
       </c>
       <c r="L25">
         <v>1</v>
@@ -2430,7 +2404,70 @@
         <v>78</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>32064</v>
+      </c>
+      <c r="D26">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="E26">
+        <v>0.6799999999999999</v>
+      </c>
+      <c r="F26">
+        <v>0.1590909090909091</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>0.8</v>
+      </c>
+      <c r="I26">
+        <v>0.03310276679841898</v>
+      </c>
+      <c r="J26">
+        <v>0.7709587204544764</v>
+      </c>
+      <c r="K26">
+        <v>0.02421500798296966</v>
+      </c>
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="M26">
+        <v>0.3378408453616634</v>
+      </c>
+      <c r="N26">
+        <v>0.05254515599343185</v>
+      </c>
+      <c r="O26">
+        <v>0.5</v>
+      </c>
+      <c r="P26">
+        <v>0.5763736263736263</v>
+      </c>
+      <c r="Q26">
+        <v>0.5</v>
+      </c>
+      <c r="R26">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="S26">
+        <v>1</v>
+      </c>
+      <c r="T26">
+        <v>1</v>
+      </c>
+      <c r="U26">
+        <v>0.2</v>
+      </c>
+      <c r="V26">
+        <v>0.3904262308715901</v>
+      </c>
+      <c r="W26">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="X26">
+        <v>0.9166666666666666</v>
       </c>
     </row>
     <row r="27" spans="1:24">
@@ -2459,13 +2496,13 @@
         <v>1</v>
       </c>
       <c r="I27">
-        <v>0.09207076378517919</v>
+        <v>0.02740740740740741</v>
       </c>
       <c r="J27">
         <v>0.4025989647388759</v>
       </c>
       <c r="K27">
-        <v>0.4416008265517827</v>
+        <v>0.2154129944660791</v>
       </c>
       <c r="L27">
         <v>1</v>
@@ -2533,13 +2570,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="I28">
-        <v>0.0469132697555353</v>
+        <v>0.02471910112359551</v>
       </c>
       <c r="J28">
         <v>0.3654064924292672</v>
       </c>
       <c r="K28">
-        <v>0.01933053453296022</v>
+        <v>0.02985817367504354</v>
       </c>
       <c r="L28">
         <v>1</v>
@@ -2607,13 +2644,13 @@
         <v>1</v>
       </c>
       <c r="I29">
-        <v>0.2455094028476227</v>
+        <v>0.09776536312849161</v>
       </c>
       <c r="J29">
         <v>0.1962583092901989</v>
       </c>
       <c r="K29">
-        <v>0.3091916087160616</v>
+        <v>0.1557653405259609</v>
       </c>
       <c r="L29">
         <v>1</v>
@@ -2681,13 +2718,13 @@
         <v>0</v>
       </c>
       <c r="I30">
-        <v>0.1511481640803845</v>
+        <v>0.07524752475247524</v>
       </c>
       <c r="J30">
         <v>0.0924350195491502</v>
       </c>
       <c r="K30">
-        <v>0.07579237102258375</v>
+        <v>0.1152213462704669</v>
       </c>
       <c r="L30">
         <v>1</v>
@@ -2755,7 +2792,7 @@
         <v>1</v>
       </c>
       <c r="I31">
-        <v>0.04231253603823304</v>
+        <v>0.05008077544426495</v>
       </c>
       <c r="J31">
         <v>0.4294028012067572</v>

</xml_diff>